<commit_message>
added chitipata in investments
</commit_message>
<xml_diff>
--- a/Finance Handling.xlsx
+++ b/Finance Handling.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThirupathireddyBijja\Documents\ibm documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThirupathireddyBijja\Documents\GithubPersonal\Standalone-Projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2FA45F0-E91E-4F0A-91C3-6023F83F90FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F901C01F-A55A-4780-933D-6E20E44E59E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Savings" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="55">
   <si>
     <t>NOTES</t>
   </si>
@@ -173,6 +173,33 @@
   </si>
   <si>
     <t xml:space="preserve">Sandeep </t>
+  </si>
+  <si>
+    <t>ChittiPata</t>
+  </si>
+  <si>
+    <t>pata amount</t>
+  </si>
+  <si>
+    <t>3 lakhs</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>15 months</t>
+  </si>
+  <si>
+    <t>left installments</t>
+  </si>
+  <si>
+    <t>advance from pd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">paid installments/amount paid </t>
+  </si>
+  <si>
+    <t>1 / 16330</t>
   </si>
 </sst>
 </file>
@@ -442,25 +469,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
@@ -469,6 +488,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -824,151 +849,151 @@
       </c>
     </row>
     <row r="2" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="16" t="s">
         <v>9</v>
       </c>
       <c r="F2" s="4"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="13">
+      <c r="D3" s="10">
         <v>1.5</v>
       </c>
-      <c r="E3" s="22"/>
+      <c r="E3" s="18"/>
       <c r="F3" s="5"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="13">
         <v>45571</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="10">
         <v>1.5</v>
       </c>
-      <c r="E4" s="22"/>
+      <c r="E4" s="18"/>
       <c r="F4" s="5"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="11">
         <v>50000</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="13">
         <v>45664</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="10">
         <v>1.5</v>
       </c>
-      <c r="E5" s="22"/>
+      <c r="E5" s="18"/>
       <c r="F5" s="5"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="10">
         <v>1.5</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="18" t="s">
         <v>12</v>
       </c>
       <c r="F6" s="5"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A7" s="21"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="22"/>
+      <c r="A7" s="17"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="18"/>
       <c r="F7" s="5"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A8" s="21"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="22"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="18"/>
       <c r="F8" s="5"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A9" s="21"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="22"/>
+      <c r="A9" s="17"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="18"/>
       <c r="F9" s="5"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A10" s="21"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="22"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="18"/>
       <c r="F10" s="5"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A11" s="21"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="22"/>
+      <c r="A11" s="17"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="18"/>
       <c r="F11" s="5"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A12" s="21"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="22"/>
+      <c r="A12" s="17"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="18"/>
       <c r="F12" s="5"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A13" s="21"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="22"/>
+      <c r="A13" s="17"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="18"/>
       <c r="F13" s="5"/>
     </row>
     <row r="14" spans="1:6" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="23"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="25"/>
+      <c r="A14" s="19"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="21"/>
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:6" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
@@ -976,11 +1001,11 @@
       <c r="A16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="27"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="23"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A17" s="9" t="s">
@@ -1075,7 +1100,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DFF7016-589F-4891-A0B1-0ACF9249D16E}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1089,29 +1114,29 @@
       <c r="A1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="27"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A2" s="9" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="23"/>
+    </row>
+    <row r="2" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="27" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1188,21 +1213,21 @@
       <c r="A11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="26"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="27"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A12" s="12" t="s">
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="23"/>
+    </row>
+    <row r="12" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.5">
+      <c r="A12" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="26" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1252,6 +1277,121 @@
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="8"/>
+    </row>
+    <row r="19" spans="1:4" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.5">
+      <c r="A20" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A21" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="10"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A24" s="10"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A26" s="10"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A27" s="10"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A28" s="10"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A29" s="10"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A30" s="10"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A31" s="10"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A32" s="10"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A33" s="10"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A34" s="10"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+    </row>
+    <row r="35" spans="1:4" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A35" s="6"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1272,11 +1412,11 @@
       <c r="A1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="27"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="23"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A2" s="10" t="s">
@@ -1403,8 +1543,12 @@
       <c r="F11" s="10"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.5">
-      <c r="A12" s="10"/>
-      <c r="B12" s="12"/>
+      <c r="A12" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="12">
+        <v>2000</v>
+      </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
@@ -1412,7 +1556,7 @@
     </row>
     <row r="13" spans="1:6" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="6"/>
-      <c r="B13" s="28"/>
+      <c r="B13" s="24"/>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>

</xml_diff>